<commit_message>
feat: add player upgrade config system and Excel-to-JSON exporter
</commit_message>
<xml_diff>
--- a/Assets/DataSource/Excel/Weapon.xlsx
+++ b/Assets/DataSource/Excel/Weapon.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Unity_Project\Planet_Rogue\Assets\DataSource\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC3B1ED9-F290-43C9-A10D-202097BEA653}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0804117E-4AAE-4359-AECB-F13A800BB496}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="17256" windowHeight="5496" activeTab="2" xr2:uid="{C760393A-9DA1-4E45-9B4F-66952DABA89A}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="17256" windowHeight="5496" activeTab="1" xr2:uid="{C760393A-9DA1-4E45-9B4F-66952DABA89A}"/>
   </bookViews>
   <sheets>
     <sheet name="sword" sheetId="1" r:id="rId1"/>
@@ -57,10 +57,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>serachRadius</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>projectileCount</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -70,6 +66,10 @@
   </si>
   <si>
     <t>true</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>searchRadius</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -574,13 +574,13 @@
         <v>5</v>
       </c>
       <c r="E1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" t="s">
         <v>7</v>
-      </c>
-      <c r="F1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" t="s">
-        <v>8</v>
       </c>
       <c r="H1" t="s">
         <v>6</v>
@@ -609,7 +609,7 @@
         <v>1</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -635,7 +635,7 @@
         <v>1</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
@@ -661,7 +661,7 @@
         <v>1</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
@@ -687,7 +687,7 @@
         <v>2</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
@@ -713,12 +713,13 @@
         <v>3</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -750,7 +751,7 @@
         <v>5</v>
       </c>
       <c r="G1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
fix: apply upgrade effects to gameplay systems
</commit_message>
<xml_diff>
--- a/Assets/DataSource/Excel/Weapon.xlsx
+++ b/Assets/DataSource/Excel/Weapon.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Unity_Project\Planet_Rogue\Assets\DataSource\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82321EA3-550B-478C-B880-6D9F6F3FCAA8}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96E016FD-B5B5-4FCA-80A0-9E864DAF74C1}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="17256" windowHeight="5496" activeTab="2" xr2:uid="{C760393A-9DA1-4E45-9B4F-66952DABA89A}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="17256" windowHeight="5496" activeTab="1" xr2:uid="{C760393A-9DA1-4E45-9B4F-66952DABA89A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sword" sheetId="1" r:id="rId1"/>
@@ -658,7 +658,7 @@
         <v>10</v>
       </c>
       <c r="G4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H4" s="1" t="s">
         <v>9</v>
@@ -684,7 +684,7 @@
         <v>10</v>
       </c>
       <c r="G5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H5" s="1" t="s">
         <v>9</v>
@@ -710,7 +710,7 @@
         <v>10</v>
       </c>
       <c r="G6">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H6" s="1" t="s">
         <v>9</v>

</xml_diff>

<commit_message>
feat: add save system and persist audio settings
</commit_message>
<xml_diff>
--- a/Assets/DataSource/Excel/Weapon.xlsx
+++ b/Assets/DataSource/Excel/Weapon.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Unity_Project\Planet_Rogue\Assets\DataSource\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6C7B171-757F-40B0-8D7B-F03848DB2E84}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B635DEE-C189-449B-A448-4E7A6F899C1D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="17256" windowHeight="5496" activeTab="1" xr2:uid="{C760393A-9DA1-4E45-9B4F-66952DABA89A}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="17256" windowHeight="5496" activeTab="2" xr2:uid="{C760393A-9DA1-4E45-9B4F-66952DABA89A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sword" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="12">
   <si>
     <t>level</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -70,6 +70,10 @@
   </si>
   <si>
     <t>searchRadius</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -551,7 +555,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC2C761C-2D8D-42F9-AE22-83FCC44930D0}">
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr defaultRowHeight="16.2" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="5" max="5" width="13.44140625" customWidth="1"/>
@@ -714,6 +718,11 @@
       </c>
       <c r="H6" s="1" t="s">
         <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="H13" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -771,7 +780,7 @@
         <v>3</v>
       </c>
       <c r="F2">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="G2">
         <v>3</v>
@@ -794,7 +803,7 @@
         <v>2.8</v>
       </c>
       <c r="F3">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="G3">
         <v>3</v>
@@ -817,7 +826,7 @@
         <v>2.6</v>
       </c>
       <c r="F4">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="G4">
         <v>4</v>
@@ -840,7 +849,7 @@
         <v>2.4</v>
       </c>
       <c r="F5">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="G5">
         <v>5</v>
@@ -863,7 +872,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="F6">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="G6">
         <v>8</v>

</xml_diff>

<commit_message>
fix: correct orbit weapon rotation
</commit_message>
<xml_diff>
--- a/Assets/DataSource/Excel/Weapon.xlsx
+++ b/Assets/DataSource/Excel/Weapon.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Unity_Project\Planet_Rogue\Assets\DataSource\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B635DEE-C189-449B-A448-4E7A6F899C1D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8609C390-6A65-40C1-BD54-A318A5BE7D18}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="17256" windowHeight="5496" activeTab="2" xr2:uid="{C760393A-9DA1-4E45-9B4F-66952DABA89A}"/>
   </bookViews>
@@ -780,7 +780,7 @@
         <v>3</v>
       </c>
       <c r="F2">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="G2">
         <v>3</v>
@@ -803,7 +803,7 @@
         <v>2.8</v>
       </c>
       <c r="F3">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="G3">
         <v>3</v>
@@ -826,7 +826,7 @@
         <v>2.6</v>
       </c>
       <c r="F4">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="G4">
         <v>4</v>
@@ -849,7 +849,7 @@
         <v>2.4</v>
       </c>
       <c r="F5">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="G5">
         <v>5</v>
@@ -872,7 +872,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="F6">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="G6">
         <v>8</v>
@@ -881,5 +881,6 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>